<commit_message>
US-15129 [PROGRESS] MSR: Adding XLSX reports
Signed-off-by: Dorian Kemps <dk@tempo-consulting.fr>
</commit_message>
<xml_diff>
--- a/bin/addons/mission_stock/report/mission_stock_report.xlsx
+++ b/bin/addons/mission_stock/report/mission_stock_report.xlsx
@@ -169,7 +169,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mmm/yyyy\ hh:mm"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="0.00000"/>
+    <numFmt numFmtId="169" formatCode="0.00###"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -257,10 +257,10 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -838,7 +838,7 @@
         <v>27</v>
       </c>
       <c r="G6" s="9">
-        <v>1</v>
+        <v>1.123456789</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>28</v>
@@ -1131,7 +1131,7 @@
         <v>27</v>
       </c>
       <c r="G11" s="10">
-        <v>1</v>
+        <v>1.1234500000000001</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>28</v>

</xml_diff>